<commit_message>
Robust download: HTTP Range resume + retry on broken connections; cache files to data/ ; toolkit never crashes on one bad file
</commit_message>
<xml_diff>
--- a/out/summary.xlsx
+++ b/out/summary.xlsx
@@ -503,10 +503,10 @@
         <v>297.9</v>
       </c>
       <c r="G2" t="n">
-        <v>293.9725353535354</v>
+        <v>293.9580202020202</v>
       </c>
       <c r="H2" t="n">
-        <v>2.304343776143029</v>
+        <v>2.311487522191812</v>
       </c>
       <c r="I2" t="n">
         <v>39600</v>
@@ -540,10 +540,10 @@
         <v>297.9</v>
       </c>
       <c r="G3" t="n">
-        <v>293.9520454545454</v>
+        <v>293.9391237373737</v>
       </c>
       <c r="H3" t="n">
-        <v>2.3069734771333</v>
+        <v>2.316382016487182</v>
       </c>
       <c r="I3" t="n">
         <v>39600</v>

</xml_diff>

<commit_message>
Auto-retry login on 429 (--wait-minutes) + graceful error message
</commit_message>
<xml_diff>
--- a/out/summary.xlsx
+++ b/out/summary.xlsx
@@ -503,10 +503,10 @@
         <v>297.9</v>
       </c>
       <c r="G2" t="n">
-        <v>293.9580202020202</v>
+        <v>293.9742828282828</v>
       </c>
       <c r="H2" t="n">
-        <v>2.311487522191812</v>
+        <v>2.311519514402313</v>
       </c>
       <c r="I2" t="n">
         <v>39600</v>
@@ -540,10 +540,10 @@
         <v>297.9</v>
       </c>
       <c r="G3" t="n">
-        <v>293.9391237373737</v>
+        <v>293.9550404040405</v>
       </c>
       <c r="H3" t="n">
-        <v>2.316382016487182</v>
+        <v>2.309405526809096</v>
       </c>
       <c r="I3" t="n">
         <v>39600</v>

</xml_diff>

<commit_message>
toolkit v2: real INSAT-3DR L2B SST structure support (2D lat/lon, fill mask, K->degC), region crop, pcolormesh maps
</commit_message>
<xml_diff>
--- a/out/summary.xlsx
+++ b/out/summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,42 +436,62 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>satellite</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>acq_start</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>units</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>shape</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>valid_pixels</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>coverage_%</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>min</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>max</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>mean</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>std</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>valid_pixels</t>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>median</t>
         </is>
       </c>
     </row>
@@ -483,33 +503,49 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>INSAT-3DR</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>01-SEP-2026T06:45:43</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>SST</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>(180, 220)</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>290</v>
-      </c>
-      <c r="F2" t="n">
-        <v>297.9</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>degC</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>(704, 700)</t>
+        </is>
       </c>
       <c r="G2" t="n">
-        <v>293.9742828282828</v>
+        <v>9880</v>
       </c>
       <c r="H2" t="n">
-        <v>2.311519514402313</v>
+        <v>2</v>
       </c>
       <c r="I2" t="n">
-        <v>39600</v>
+        <v>24.06862792968752</v>
+      </c>
+      <c r="J2" t="n">
+        <v>33.58846435546877</v>
+      </c>
+      <c r="K2" t="n">
+        <v>29.40537791387275</v>
+      </c>
+      <c r="L2" t="n">
+        <v>2.333731979662678</v>
+      </c>
+      <c r="M2" t="n">
+        <v>29.70713195800784</v>
       </c>
     </row>
     <row r="3">
@@ -520,33 +556,49 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>INSAT-3DR</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>01-SEP-2026T07:45:43</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>SST</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>(180, 220)</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>290</v>
-      </c>
-      <c r="F3" t="n">
-        <v>297.9</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>degC</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>(704, 700)</t>
+        </is>
       </c>
       <c r="G3" t="n">
-        <v>293.9550404040405</v>
+        <v>9880</v>
       </c>
       <c r="H3" t="n">
-        <v>2.309405526809096</v>
+        <v>2</v>
       </c>
       <c r="I3" t="n">
-        <v>39600</v>
+        <v>24.1203552246094</v>
+      </c>
+      <c r="J3" t="n">
+        <v>33.5921569824219</v>
+      </c>
+      <c r="K3" t="n">
+        <v>29.39924899267284</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2.343880336202431</v>
+      </c>
+      <c r="M3" t="n">
+        <v>29.68491516113284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Map polish: land/no-data background + darker spines
</commit_message>
<xml_diff>
--- a/out/summary.xlsx
+++ b/out/summary.xlsx
@@ -533,19 +533,19 @@
         <v>2</v>
       </c>
       <c r="I2" t="n">
-        <v>24.06862792968752</v>
+        <v>24.10030517578127</v>
       </c>
       <c r="J2" t="n">
-        <v>33.58846435546877</v>
+        <v>33.56258544921877</v>
       </c>
       <c r="K2" t="n">
-        <v>29.40537791387275</v>
+        <v>29.41254147981345</v>
       </c>
       <c r="L2" t="n">
-        <v>2.333731979662678</v>
+        <v>2.345193955561933</v>
       </c>
       <c r="M2" t="n">
-        <v>29.70713195800784</v>
+        <v>29.69643554687502</v>
       </c>
     </row>
     <row r="3">
@@ -586,19 +586,19 @@
         <v>2</v>
       </c>
       <c r="I3" t="n">
-        <v>24.1203552246094</v>
+        <v>24.12090454101565</v>
       </c>
       <c r="J3" t="n">
-        <v>33.5921569824219</v>
+        <v>33.5623718261719</v>
       </c>
       <c r="K3" t="n">
-        <v>29.39924899267284</v>
+        <v>29.41246245225916</v>
       </c>
       <c r="L3" t="n">
-        <v>2.343880336202431</v>
+        <v>2.353302795975066</v>
       </c>
       <c r="M3" t="n">
-        <v>29.68491516113284</v>
+        <v>29.6975036621094</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MATSYA agentic layer: 6-agent DAG (supervisor/ocean/risk/nav/policy/synth), tactical command UI, live server, audit log
</commit_message>
<xml_diff>
--- a/out/summary.xlsx
+++ b/out/summary.xlsx
@@ -832,12 +832,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SST (thermal fronts, PFZ)</t>
+          <t>SST (fronts + PFZ)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ISRO MOSDAC (INSAT-3DR IMAGER)</t>
+          <t>ISRO MOSDAC (INSAT-3DR)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -864,12 +864,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sea surface wind (safety)</t>
+          <t>Sea wind (safety)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ISRO MOSDAC (INSAT-3DR IMAGER)</t>
+          <t>ISRO MOSDAC (INSAT-3DR)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MarineRegions / VLIZ (EEZ v12)</t>
+          <t>MarineRegions / VLIZ</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -933,7 +933,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Natural Earth (public domain)</t>
+          <t>Natural Earth</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MOSDAC API me maujood NAHI</t>
+          <t>MOSDAC API me NAHI</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">

</xml_diff>